<commit_message>
Creacion de agente para descuento
</commit_message>
<xml_diff>
--- a/Descuentos/Productos.xlsx
+++ b/Descuentos/Productos.xlsx
@@ -1081,13 +1081,13 @@
         </is>
       </c>
       <c r="D11" s="42" t="n">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E11" s="42" t="n">
         <v>-1</v>
       </c>
       <c r="F11" s="43" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G11" s="38" t="n"/>
       <c r="H11" s="38" t="n"/>
@@ -1305,13 +1305,13 @@
         </is>
       </c>
       <c r="D18" s="42" t="n">
-        <v>252</v>
+        <v>238</v>
       </c>
       <c r="E18" s="42" t="n">
-        <v>-8</v>
+        <v>-6</v>
       </c>
       <c r="F18" s="43" t="n">
-        <v>244</v>
+        <v>232</v>
       </c>
       <c r="G18" s="38" t="n"/>
       <c r="H18" s="38" t="n"/>
@@ -2337,13 +2337,13 @@
         </is>
       </c>
       <c r="D49" s="42" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E49" s="42" t="n">
         <v>-1</v>
       </c>
       <c r="F49" s="43" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G49" s="38" t="n"/>
       <c r="H49" s="38" t="n"/>
@@ -4157,13 +4157,13 @@
         </is>
       </c>
       <c r="D105" s="42" t="n">
-        <v>0</v>
+        <v>-24</v>
       </c>
       <c r="E105" s="42" t="n">
         <v>-12</v>
       </c>
       <c r="F105" s="43" t="n">
-        <v>-12</v>
+        <v>-36</v>
       </c>
       <c r="G105" s="38" t="n"/>
       <c r="H105" s="38" t="n"/>
@@ -4225,13 +4225,13 @@
         </is>
       </c>
       <c r="D107" s="42" t="n">
-        <v>7</v>
+        <v>-17</v>
       </c>
       <c r="E107" s="42" t="n">
         <v>-12</v>
       </c>
       <c r="F107" s="43" t="n">
-        <v>-5</v>
+        <v>-29</v>
       </c>
       <c r="G107" s="38" t="n"/>
       <c r="H107" s="38" t="n"/>
@@ -4519,13 +4519,13 @@
         </is>
       </c>
       <c r="D116" s="42" t="n">
-        <v>-83</v>
+        <v>-155</v>
       </c>
       <c r="E116" s="42" t="n">
         <v>-36</v>
       </c>
       <c r="F116" s="43" t="n">
-        <v>-119</v>
+        <v>-191</v>
       </c>
       <c r="G116" s="38" t="n"/>
       <c r="H116" s="38" t="n"/>
@@ -6139,13 +6139,13 @@
         </is>
       </c>
       <c r="D166" s="42" t="n">
-        <v>119</v>
+        <v>95</v>
       </c>
       <c r="E166" s="42" t="n">
         <v>-12</v>
       </c>
       <c r="F166" s="43" t="n">
-        <v>107</v>
+        <v>83</v>
       </c>
       <c r="G166" s="38" t="n"/>
       <c r="H166" s="38" t="n"/>
@@ -6567,13 +6567,13 @@
         </is>
       </c>
       <c r="D179" s="42" t="n">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="E179" s="42" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="F179" s="43" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="G179" s="38" t="n"/>
       <c r="H179" s="38" t="n"/>
@@ -6839,13 +6839,13 @@
         </is>
       </c>
       <c r="D187" s="42" t="n">
-        <v>1</v>
+        <v>-28</v>
       </c>
       <c r="E187" s="42" t="n">
-        <v>-15</v>
+        <v>-14</v>
       </c>
       <c r="F187" s="43" t="n">
-        <v>-14</v>
+        <v>-42</v>
       </c>
       <c r="G187" s="38" t="n"/>
       <c r="H187" s="38" t="n"/>
@@ -7171,13 +7171,13 @@
         </is>
       </c>
       <c r="D197" s="42" t="n">
-        <v>101</v>
+        <v>80</v>
       </c>
       <c r="E197" s="42" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="F197" s="43" t="n">
-        <v>90</v>
+        <v>70</v>
       </c>
       <c r="G197" s="38" t="n"/>
       <c r="H197" s="38" t="n"/>
@@ -7491,13 +7491,13 @@
         </is>
       </c>
       <c r="D207" s="42" t="n">
-        <v>43</v>
+        <v>3</v>
       </c>
       <c r="E207" s="42" t="n">
         <v>-20</v>
       </c>
       <c r="F207" s="43" t="n">
-        <v>23</v>
+        <v>-17</v>
       </c>
       <c r="G207" s="38" t="n"/>
       <c r="H207" s="38" t="n"/>
@@ -7763,13 +7763,13 @@
         </is>
       </c>
       <c r="D215" s="42" t="n">
-        <v>31</v>
+        <v>-9</v>
       </c>
       <c r="E215" s="42" t="n">
         <v>-20</v>
       </c>
       <c r="F215" s="43" t="n">
-        <v>11</v>
+        <v>-29</v>
       </c>
       <c r="G215" s="38" t="n"/>
       <c r="H215" s="38" t="n"/>
@@ -9343,13 +9343,13 @@
         </is>
       </c>
       <c r="D263" s="42" t="n">
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="E263" s="42" t="n">
-        <v>-8</v>
+        <v>-7</v>
       </c>
       <c r="F263" s="43" t="n">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="G263" s="38" t="n"/>
       <c r="H263" s="38" t="n"/>
@@ -9443,13 +9443,13 @@
         </is>
       </c>
       <c r="D266" s="42" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E266" s="42" t="n">
         <v>-1</v>
       </c>
       <c r="F266" s="43" t="n">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="G266" s="38" t="n"/>
       <c r="H266" s="38" t="n"/>
@@ -10393,13 +10393,13 @@
         </is>
       </c>
       <c r="D296" s="45" t="n">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="E296" s="45" t="n">
         <v>-2</v>
       </c>
       <c r="F296" s="43" t="n">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="G296" s="38" t="n"/>
       <c r="H296" s="38" t="n"/>
@@ -10439,13 +10439,13 @@
         </is>
       </c>
       <c r="D297" s="45" t="n">
-        <v>894</v>
+        <v>890</v>
       </c>
       <c r="E297" s="45" t="n">
         <v>-2</v>
       </c>
       <c r="F297" s="43" t="n">
-        <v>892</v>
+        <v>888</v>
       </c>
       <c r="G297" s="38" t="n"/>
       <c r="H297" s="38" t="n"/>
@@ -10507,13 +10507,13 @@
         </is>
       </c>
       <c r="D299" s="45" t="n">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="E299" s="45" t="n">
         <v>-2</v>
       </c>
       <c r="F299" s="43" t="n">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="G299" s="38" t="n"/>
       <c r="H299" s="38" t="n"/>
@@ -10923,13 +10923,13 @@
         </is>
       </c>
       <c r="D311" s="45" t="n">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="E311" s="45" t="n">
         <v>-2</v>
       </c>
       <c r="F311" s="43" t="n">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="G311" s="38" t="n"/>
       <c r="H311" s="38" t="n"/>
@@ -10959,13 +10959,13 @@
         </is>
       </c>
       <c r="D312" s="45" t="n">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E312" s="45" t="n">
         <v>-2</v>
       </c>
       <c r="F312" s="43" t="n">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="G312" s="38" t="n"/>
       <c r="H312" s="38" t="n"/>
@@ -11713,13 +11713,13 @@
         </is>
       </c>
       <c r="D337" s="45" t="n">
-        <v>-9</v>
+        <v>-15</v>
       </c>
       <c r="E337" s="45" t="n">
         <v>-3</v>
       </c>
       <c r="F337" s="43" t="n">
-        <v>-12</v>
+        <v>-18</v>
       </c>
       <c r="G337" s="38" t="n"/>
       <c r="H337" s="38" t="n"/>
@@ -11989,13 +11989,13 @@
         </is>
       </c>
       <c r="D346" s="45" t="n">
-        <v>-9</v>
+        <v>-15</v>
       </c>
       <c r="E346" s="45" t="n">
         <v>-3</v>
       </c>
       <c r="F346" s="43" t="n">
-        <v>-12</v>
+        <v>-18</v>
       </c>
       <c r="G346" s="38" t="n"/>
       <c r="H346" s="38" t="n"/>
@@ -12085,13 +12085,13 @@
         </is>
       </c>
       <c r="D349" s="45" t="n">
-        <v>-6</v>
+        <v>-10</v>
       </c>
       <c r="E349" s="45" t="n">
         <v>-2</v>
       </c>
       <c r="F349" s="43" t="n">
-        <v>-8</v>
+        <v>-12</v>
       </c>
       <c r="G349" s="38" t="n"/>
       <c r="H349" s="38" t="n"/>
@@ -12211,13 +12211,13 @@
         </is>
       </c>
       <c r="D353" s="45" t="n">
-        <v>-6</v>
+        <v>-10</v>
       </c>
       <c r="E353" s="45" t="n">
         <v>-2</v>
       </c>
       <c r="F353" s="43" t="n">
-        <v>-8</v>
+        <v>-12</v>
       </c>
       <c r="G353" s="38" t="n"/>
       <c r="H353" s="38" t="n"/>
@@ -12307,13 +12307,13 @@
         </is>
       </c>
       <c r="D356" s="45" t="n">
-        <v>-9</v>
+        <v>-15</v>
       </c>
       <c r="E356" s="45" t="n">
         <v>-3</v>
       </c>
       <c r="F356" s="43" t="n">
-        <v>-12</v>
+        <v>-18</v>
       </c>
       <c r="G356" s="38" t="n"/>
       <c r="H356" s="38" t="n"/>
@@ -12523,13 +12523,13 @@
         </is>
       </c>
       <c r="D363" s="45" t="n">
-        <v>-6</v>
+        <v>-10</v>
       </c>
       <c r="E363" s="45" t="n">
         <v>-2</v>
       </c>
       <c r="F363" s="43" t="n">
-        <v>-8</v>
+        <v>-12</v>
       </c>
       <c r="G363" s="38" t="n"/>
       <c r="H363" s="38" t="n"/>

</xml_diff>